<commit_message>
Correct rice tariff-cut date and tighten data sources
- EO 62 tariff cut dated 5 Jul 2024 (was 1 Jul); events name EO 62, 93, 105
- Specific source links for NCR-25 wage order and rice policy events
- Re-extracted raw workbook and rebuilt dashboard and download zip
- Remove stray .DS_Store from powerbi/
</commit_message>
<xml_diff>
--- a/raw/ph_food_economy_raw.xlsx
+++ b/raw/ph_food_economy_raw.xlsx
@@ -4599,7 +4599,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-24T16:26:57+00:00</t>
+          <t>2026-10-25T18:22:22+00:00</t>
         </is>
       </c>
     </row>
@@ -19967,7 +19967,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>https://nwpc.dole.gov.ph/regionandwages/current-real-minimum-wage-rates/</t>
+          <t>https://www.pna.gov.ph/articles/1227990</t>
         </is>
       </c>
     </row>
@@ -20045,7 +20045,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2024-07-01</t>
+          <t>2024-07-05</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -20055,7 +20055,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://www.da.gov.ph/rice-import-ban-lifts-palay-prices-nationwide/</t>
+          <t>https://portcalls.com/marcos-issues-eo-62-modifying-import-tariffs-including-on-rice</t>
         </is>
       </c>
     </row>
@@ -20067,12 +20067,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Imports of regular and well-milled rice suspended</t>
+          <t>Imports of regular and well-milled rice suspended (EO 93)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://www.da.gov.ph/rice-import-ban-lifts-palay-prices-nationwide/</t>
+          <t>https://portcalls.com/ph-rice-import-ban-extended-to-end-2025/</t>
         </is>
       </c>
     </row>
@@ -20084,7 +20084,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Price-indexed rice tariff (15-35%) starts; imports resume</t>
+          <t>Price-indexed rice tariff (15-35%) starts; imports resume (EO 105)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">

</xml_diff>

<commit_message>
Update FX with provisional Oct 2026 peso rate and refit dollar forecast
- extract_data.py: add current month-to-date USD/PHP from ECB daily rates (marked PROVISIONAL)
- clean_reference.py: write data/fx_monthly.csv with provisional flag, plus self-checks
- dashboard: forecast fitted on fx_monthly (Dec 2026: P63.62, range P62.53-64.70); Oct to-date shown
- check_project.py: FX consistency checks (nat vs fx, provisional rows, jumps, forecast wiring)
- README: latest peso figures

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/raw/ph_food_economy_raw.xlsx
+++ b/raw/ph_food_economy_raw.xlsx
@@ -4599,7 +4599,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-25T18:22:22+00:00</t>
+          <t>2026-10-26T22:26:35+00:00</t>
         </is>
       </c>
     </row>
@@ -17907,7 +17907,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E67"/>
+  <dimension ref="A1:E69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19716,6 +19716,60 @@
       <c r="E67" t="inlineStr">
         <is>
           <t>US dollar/Euro ECB reference exchange rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>PHP</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>70.6737</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>PROVISIONAL: average of ECB daily reference rates to 2026-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>1.1214</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>PROVISIONAL: average of ECB daily reference rates to 2026-10-26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add BSP outlook (policy rate 5.5%, 2026 inflation forecast 6.1%) and refresh live data
October CPI not yet released by PSA (due early November).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/raw/ph_food_economy_raw.xlsx
+++ b/raw/ph_food_economy_raw.xlsx
@@ -16,8 +16,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sws_hunger" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ncr_min_wage" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rice_policy_events" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="region_lookup" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="about" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="bsp_outlook" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="region_lookup" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="about" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4577,546 +4578,88 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>region_key</t>
+          <t>date</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>region</t>
+          <t>item</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>island_group</t>
+          <t>value</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>rice_label</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>cpi_label</t>
+          <t>source</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PH</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Philippines</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>National</t>
-        </is>
+          <t>policy_rate_pct</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>5.5</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Philippines</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>PHILIPPINES</t>
+          <t>https://www.manilatimes.net/2026/10/27/business/top-business/inflation-threatens-prolonged-tightening/2454325</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>NCR</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NCR</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Luzon</t>
-        </is>
+          <t>inflation_forecast_2026_pct</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>6.1</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NCR - National Capital Region</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>National Capital Region (NCR)</t>
+          <t>https://www.manilatimes.net/2026/10/27/business/top-business/inflation-threatens-prolonged-tightening/2454325</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CAR</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CAR</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Luzon</t>
-        </is>
+          <t>inflation_forecast_2027_pct</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>6</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>CAR - Cordillera Administrative Region</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Cordillera Administrative Region (CAR)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>R01</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Ilocos</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Luzon</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>I - Ilocos Region</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Region I (Ilocos Region)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>R02</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Cagayan Valley</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Luzon</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>II - Cagayan Valley</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Region II (Cagayan Valley)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>R03</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Central Luzon</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Luzon</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>III - Central Luzon</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Region III (Central Luzon)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>R4A</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>CALABARZON</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Luzon</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>IV-A - CALABARZON</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Region IV-A (CALABARZON)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>R4B</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>MIMAROPA</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Luzon</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>MIMAROPA Region</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>MIMAROPA Region</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>R05</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Bicol</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Luzon</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>V - Bicol Region</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Region V (Bicol Region)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>R06</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Western Visayas</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Visayas</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>VI - Western Visayas</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Region VI (Western Visayas)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>NIR</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Negros Island</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Visayas</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Negros Island Region (NIR)</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Negros Island Region (NIR)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>R07</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Central Visayas</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Visayas</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>VII - Central Visayas</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Region VII (Central Visayas)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>R08</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Eastern Visayas</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Visayas</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>VIII - Eastern Visayas</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Region VIII (Eastern Visayas)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>R09</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Zamboanga Peninsula</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Mindanao</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>IX - Zamboanga Peninsula</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Region IX (Zamboanga Peninsula)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>R10</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Northern Mindanao</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Mindanao</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>X - Northern Mindanao</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Region X (Northern Mindanao)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>R11</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>Davao</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Mindanao</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>XI - Davao Region</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Region XI (Davao Region)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>R12</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>SOCCSKSARGEN</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Mindanao</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>XII - SOCCSKSARGEN</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Region XII (SOCCSKSARGEN)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>R13</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Caraga</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Mindanao</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>XIII - Caraga</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Region XIII (Caraga)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>BARMM</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>BARMM</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Mindanao</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>BARMM - Bangsamoro Autonomous Region in Muslim Mindanao</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Bangsamoro Autonomous Region in Muslim Mindanao (BARMM)</t>
+          <t>https://www.manilatimes.net/2026/10/27/business/top-business/inflation-threatens-prolonged-tightening/2454325</t>
         </is>
       </c>
     </row>
@@ -5131,6 +4674,560 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>region_key</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>island_group</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>rice_label</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>cpi_label</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>PH</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Philippines</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>National</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Philippines</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>PHILIPPINES</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>NCR</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Luzon</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NCR - National Capital Region</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>National Capital Region (NCR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Luzon</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>CAR - Cordillera Administrative Region</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Cordillera Administrative Region (CAR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>R01</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ilocos</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Luzon</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>I - Ilocos Region</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Region I (Ilocos Region)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>R02</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Cagayan Valley</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Luzon</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>II - Cagayan Valley</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Region II (Cagayan Valley)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>R03</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Central Luzon</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Luzon</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>III - Central Luzon</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Region III (Central Luzon)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>R4A</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>CALABARZON</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Luzon</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>IV-A - CALABARZON</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Region IV-A (CALABARZON)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>R4B</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>MIMAROPA</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Luzon</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>MIMAROPA Region</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>MIMAROPA Region</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>R05</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Bicol</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Luzon</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>V - Bicol Region</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Region V (Bicol Region)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>R06</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Western Visayas</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Visayas</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>VI - Western Visayas</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Region VI (Western Visayas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>NIR</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Negros Island</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Visayas</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Negros Island Region (NIR)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Negros Island Region (NIR)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>R07</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Central Visayas</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Visayas</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>VII - Central Visayas</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Region VII (Central Visayas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>R08</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Eastern Visayas</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Visayas</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>VIII - Eastern Visayas</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Region VIII (Eastern Visayas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>R09</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Zamboanga Peninsula</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Mindanao</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>IX - Zamboanga Peninsula</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Region IX (Zamboanga Peninsula)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>R10</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Northern Mindanao</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Mindanao</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>X - Northern Mindanao</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Region X (Northern Mindanao)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>R11</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Davao</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Mindanao</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>XI - Davao Region</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Region XI (Davao Region)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>R12</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>SOCCSKSARGEN</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Mindanao</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>XII - SOCCSKSARGEN</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Region XII (SOCCSKSARGEN)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>R13</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Caraga</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Mindanao</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>XIII - Caraga</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Region XIII (Caraga)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>BARMM</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>BARMM</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Mindanao</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>BARMM - Bangsamoro Autonomous Region in Muslim Mindanao</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Bangsamoro Autonomous Region in Muslim Mindanao (BARMM)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -5154,7 +5251,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-26T22:29:18+00:00</t>
+          <t>2026-10-27T04:54:45+00:00</t>
         </is>
       </c>
     </row>

</xml_diff>